<commit_message>
Progreso hasta parte C
</commit_message>
<xml_diff>
--- a/Archivos_aux/Tablas modelos.xlsx
+++ b/Archivos_aux/Tablas modelos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Luis Alberto\Documents\GitHub\Analisis_data_c_de_credito\Archivos_aux\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7640981-A729-414E-8699-DCDBF387E5BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E9FC4B2-CF69-4331-8739-68DA7034E1A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4230" yWindow="3195" windowWidth="15375" windowHeight="8325" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="10245" windowHeight="11520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Modelo1" sheetId="1" r:id="rId1"/>
@@ -91,7 +91,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -114,6 +117,13 @@
       <sz val="11"/>
       <color rgb="FFC00000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -166,10 +176,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -195,9 +206,11 @@
     <xf numFmtId="10" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -497,7 +510,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="57" customWidth="1"/>
@@ -507,7 +520,7 @@
     <col min="7" max="7" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -530,7 +543,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -552,8 +565,9 @@
       <c r="G2" s="4">
         <v>9.6000000000000002E-2</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" s="9"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
         <v>2</v>
       </c>
@@ -575,8 +589,9 @@
       <c r="G3" s="7">
         <v>7.4399999999999994E-2</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H3" s="9"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -598,8 +613,9 @@
       <c r="G4" s="4">
         <v>5.7299999999999997E-2</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H4" s="9"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -621,8 +637,9 @@
       <c r="G5" s="7">
         <v>4.24E-2</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H5" s="9"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -644,8 +661,9 @@
       <c r="G6" s="4">
         <v>3.0700000000000002E-2</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H6" s="9"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>6</v>
       </c>
@@ -667,8 +685,9 @@
       <c r="G7" s="7">
         <v>2.07E-2</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H7" s="9"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -690,8 +709,9 @@
       <c r="G8" s="4">
         <v>1.2E-2</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H8" s="9"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>8</v>
       </c>
@@ -713,8 +733,9 @@
       <c r="G9" s="7">
         <v>6.4999999999999997E-3</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H9" s="9"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -736,8 +757,9 @@
       <c r="G10" s="4">
         <v>3.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H10" s="9"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>10</v>
       </c>

</xml_diff>